<commit_message>
Publish source-free M&A checklist workbooks
</commit_message>
<xml_diff>
--- a/public/resources/MikeYe-MA-Due-Diligence-Checklist-v1.0.xlsx
+++ b/public/resources/MikeYe-MA-Due-Diligence-Checklist-v1.0.xlsx
@@ -2,11 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R28c896ad4b324dc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R9a13d7ed282f4131"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Map" sheetId="3" r:id="Rff9a1e35b37f4499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="4" r:id="R53dd27dcddf44bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R22d9ae7cc9554283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R91679f5bfd274514"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R372add6c48d14b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Map" sheetId="3" r:id="R40fb3c9651e04d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="4" r:id="Rc9c82ade736849f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -55,11 +54,6 @@
       <x:b/>
       <x:sz val="14"/>
       <x:color rgb="FF1A1A18"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF1D4E89"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -138,7 +132,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -270,12 +264,6 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -330,9 +318,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DDChecklistTable" displayName="DDChecklistTable" ref="A5:S117" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:S117"/>
-  <x:tableColumns count="19">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DDChecklistTable" displayName="DDChecklistTable" ref="A5:R117" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:R117"/>
+  <x:tableColumns count="18">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Phase"/>
     <x:tableColumn id="3" name="Workstream"/>
@@ -351,7 +339,6 @@
     <x:tableColumn id="16" name="Agreement / price action"/>
     <x:tableColumn id="17" name="Integration handoff"/>
     <x:tableColumn id="18" name="Reviewer decision"/>
-    <x:tableColumn id="19" name="Source IDs"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -404,21 +391,6 @@
     <x:tableColumn id="13" name="Due date"/>
     <x:tableColumn id="14" name="Status"/>
     <x:tableColumn id="15" name="Reviewer decision"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DiligenceSourcesTable" displayName="DiligenceSourcesTable" ref="A5:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F13"/>
-  <x:tableColumns count="6">
-    <x:tableColumn id="1" name="Source ID"/>
-    <x:tableColumn id="2" name="Organization"/>
-    <x:tableColumn id="3" name="Resource"/>
-    <x:tableColumn id="4" name="Accessed"/>
-    <x:tableColumn id="5" name="URL"/>
-    <x:tableColumn id="6" name="Use in this workbook"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -887,7 +859,6 @@
     <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2" ht="24" customHeight="1">
@@ -919,7 +890,6 @@
       <x:c r="P4" s="5"/>
       <x:c r="Q4" s="5"/>
       <x:c r="R4" s="5"/>
-      <x:c r="S4" s="5"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="50" t="str">
@@ -975,9 +945,6 @@
       </x:c>
       <x:c r="R5" s="50" t="str">
         <x:v>Reviewer decision</x:v>
-      </x:c>
-      <x:c r="S5" s="50" t="str">
-        <x:v>Source IDs</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -1025,9 +992,6 @@
       <x:c r="R6" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S6" s="51" t="str">
-        <x:v>M01;S01;S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="51" t="str">
@@ -1074,9 +1038,6 @@
       <x:c r="R7" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S7" s="51" t="str">
-        <x:v>M01;S04</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="51" t="str">
@@ -1123,9 +1084,6 @@
       <x:c r="R8" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S8" s="51" t="str">
-        <x:v>M01;S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="51" t="str">
@@ -1172,9 +1130,6 @@
       <x:c r="R9" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S9" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="51" t="str">
@@ -1221,9 +1176,6 @@
       <x:c r="R10" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S10" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="51" t="str">
@@ -1270,9 +1222,6 @@
       <x:c r="R11" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S11" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="51" t="str">
@@ -1319,9 +1268,6 @@
       <x:c r="R12" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S12" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="51" t="str">
@@ -1368,9 +1314,6 @@
       <x:c r="R13" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S13" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="51" t="str">
@@ -1417,9 +1360,6 @@
       <x:c r="R14" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S14" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="51" t="str">
@@ -1466,9 +1406,6 @@
       <x:c r="R15" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S15" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="51" t="str">
@@ -1515,9 +1452,6 @@
       <x:c r="R16" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S16" s="51" t="str">
-        <x:v>M01;S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="51" t="str">
@@ -1564,9 +1498,6 @@
       <x:c r="R17" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S17" s="51" t="str">
-        <x:v>M01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="51" t="str">
@@ -1613,9 +1544,6 @@
       <x:c r="R18" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S18" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="51" t="str">
@@ -1662,9 +1590,6 @@
       <x:c r="R19" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S19" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="51" t="str">
@@ -1711,9 +1636,6 @@
       <x:c r="R20" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S20" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="51" t="str">
@@ -1760,9 +1682,6 @@
       <x:c r="R21" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S21" s="51" t="str">
-        <x:v>S03;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="51" t="str">
@@ -1809,9 +1728,6 @@
       <x:c r="R22" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S22" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="51" t="str">
@@ -1858,9 +1774,6 @@
       <x:c r="R23" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S23" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="51" t="str">
@@ -1907,9 +1820,6 @@
       <x:c r="R24" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S24" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="51" t="str">
@@ -1956,9 +1866,6 @@
       <x:c r="R25" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S25" s="51" t="str">
-        <x:v>M01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="51" t="str">
@@ -2005,9 +1912,6 @@
       <x:c r="R26" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S26" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="51" t="str">
@@ -2054,9 +1958,6 @@
       <x:c r="R27" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S27" s="51" t="str">
-        <x:v>S03;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="51" t="str">
@@ -2103,9 +2004,6 @@
       <x:c r="R28" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S28" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="51" t="str">
@@ -2152,9 +2050,6 @@
       <x:c r="R29" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S29" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="51" t="str">
@@ -2201,9 +2096,6 @@
       <x:c r="R30" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S30" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="51" t="str">
@@ -2250,9 +2142,6 @@
       <x:c r="R31" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S31" s="51" t="str">
-        <x:v>M01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="51" t="str">
@@ -2299,9 +2188,6 @@
       <x:c r="R32" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S32" s="51" t="str">
-        <x:v>S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="51" t="str">
@@ -2348,9 +2234,6 @@
       <x:c r="R33" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S33" s="51" t="str">
-        <x:v>S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="51" t="str">
@@ -2397,9 +2280,6 @@
       <x:c r="R34" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S34" s="51" t="str">
-        <x:v>S02;S04;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="51" t="str">
@@ -2446,9 +2326,6 @@
       <x:c r="R35" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S35" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="51" t="str">
@@ -2495,9 +2372,6 @@
       <x:c r="R36" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S36" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="51" t="str">
@@ -2544,9 +2418,6 @@
       <x:c r="R37" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S37" s="51" t="str">
-        <x:v>M01;S04</x:v>
-      </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="51" t="str">
@@ -2593,9 +2464,6 @@
       <x:c r="R38" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S38" s="51" t="str">
-        <x:v>S02;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="51" t="str">
@@ -2642,9 +2510,6 @@
       <x:c r="R39" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S39" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="51" t="str">
@@ -2691,9 +2556,6 @@
       <x:c r="R40" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S40" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="51" t="str">
@@ -2740,9 +2602,6 @@
       <x:c r="R41" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S41" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="51" t="str">
@@ -2789,9 +2648,6 @@
       <x:c r="R42" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S42" s="51" t="str">
-        <x:v>M01;S04</x:v>
-      </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="51" t="str">
@@ -2838,9 +2694,6 @@
       <x:c r="R43" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S43" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="51" t="str">
@@ -2887,9 +2740,6 @@
       <x:c r="R44" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S44" s="51" t="str">
-        <x:v>M01;S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="51" t="str">
@@ -2936,9 +2786,6 @@
       <x:c r="R45" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S45" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="51" t="str">
@@ -2985,9 +2832,6 @@
       <x:c r="R46" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S46" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="51" t="str">
@@ -3034,9 +2878,6 @@
       <x:c r="R47" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S47" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="51" t="str">
@@ -3083,9 +2924,6 @@
       <x:c r="R48" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S48" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="51" t="str">
@@ -3132,9 +2970,6 @@
       <x:c r="R49" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S49" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="51" t="str">
@@ -3181,9 +3016,6 @@
       <x:c r="R50" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S50" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="51" t="str">
@@ -3230,9 +3062,6 @@
       <x:c r="R51" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S51" s="51" t="str">
-        <x:v>S03;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
       <x:c r="A52" s="51" t="str">
@@ -3279,9 +3108,6 @@
       <x:c r="R52" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S52" s="51" t="str">
-        <x:v>S01;S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
       <x:c r="A53" s="51" t="str">
@@ -3328,9 +3154,6 @@
       <x:c r="R53" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S53" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
       <x:c r="A54" s="51" t="str">
@@ -3377,9 +3200,6 @@
       <x:c r="R54" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S54" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
       <x:c r="A55" s="51" t="str">
@@ -3426,9 +3246,6 @@
       <x:c r="R55" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S55" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
       <x:c r="A56" s="51" t="str">
@@ -3475,9 +3292,6 @@
       <x:c r="R56" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S56" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
       <x:c r="A57" s="51" t="str">
@@ -3524,9 +3338,6 @@
       <x:c r="R57" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S57" s="51" t="str">
-        <x:v>M01;S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
       <x:c r="A58" s="51" t="str">
@@ -3573,9 +3384,6 @@
       <x:c r="R58" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S58" s="51" t="str">
-        <x:v>M01;S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
       <x:c r="A59" s="51" t="str">
@@ -3622,9 +3430,6 @@
       <x:c r="R59" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S59" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
       <x:c r="A60" s="51" t="str">
@@ -3671,9 +3476,6 @@
       <x:c r="R60" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S60" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
       <x:c r="A61" s="51" t="str">
@@ -3720,9 +3522,6 @@
       <x:c r="R61" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S61" s="51" t="str">
-        <x:v>S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="62" ht="42" customHeight="1">
       <x:c r="A62" s="51" t="str">
@@ -3769,9 +3568,6 @@
       <x:c r="R62" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S62" s="51" t="str">
-        <x:v>S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
       <x:c r="A63" s="51" t="str">
@@ -3818,9 +3614,6 @@
       <x:c r="R63" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S63" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="64" ht="42" customHeight="1">
       <x:c r="A64" s="51" t="str">
@@ -3867,9 +3660,6 @@
       <x:c r="R64" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S64" s="51" t="str">
-        <x:v>M01;S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="65" ht="42" customHeight="1">
       <x:c r="A65" s="51" t="str">
@@ -3916,9 +3706,6 @@
       <x:c r="R65" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S65" s="51" t="str">
-        <x:v>S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="66" ht="42" customHeight="1">
       <x:c r="A66" s="51" t="str">
@@ -3965,9 +3752,6 @@
       <x:c r="R66" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S66" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="67" ht="42" customHeight="1">
       <x:c r="A67" s="51" t="str">
@@ -4014,9 +3798,6 @@
       <x:c r="R67" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S67" s="51" t="str">
-        <x:v>S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="68" ht="42" customHeight="1">
       <x:c r="A68" s="51" t="str">
@@ -4063,9 +3844,6 @@
       <x:c r="R68" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S68" s="51" t="str">
-        <x:v>S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="69" ht="42" customHeight="1">
       <x:c r="A69" s="51" t="str">
@@ -4112,9 +3890,6 @@
       <x:c r="R69" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S69" s="51" t="str">
-        <x:v>S03;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
       <x:c r="A70" s="51" t="str">
@@ -4161,9 +3936,6 @@
       <x:c r="R70" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S70" s="51" t="str">
-        <x:v>S03;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="71" ht="42" customHeight="1">
       <x:c r="A71" s="51" t="str">
@@ -4210,9 +3982,6 @@
       <x:c r="R71" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S71" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="72" ht="42" customHeight="1">
       <x:c r="A72" s="51" t="str">
@@ -4259,9 +4028,6 @@
       <x:c r="R72" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S72" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
       <x:c r="A73" s="51" t="str">
@@ -4308,9 +4074,6 @@
       <x:c r="R73" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S73" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="74" ht="42" customHeight="1">
       <x:c r="A74" s="51" t="str">
@@ -4357,9 +4120,6 @@
       <x:c r="R74" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S74" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="75" ht="42" customHeight="1">
       <x:c r="A75" s="51" t="str">
@@ -4406,9 +4166,6 @@
       <x:c r="R75" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S75" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="76" ht="42" customHeight="1">
       <x:c r="A76" s="51" t="str">
@@ -4455,9 +4212,6 @@
       <x:c r="R76" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S76" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="77" ht="42" customHeight="1">
       <x:c r="A77" s="51" t="str">
@@ -4504,9 +4258,6 @@
       <x:c r="R77" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S77" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="78" ht="42" customHeight="1">
       <x:c r="A78" s="51" t="str">
@@ -4553,9 +4304,6 @@
       <x:c r="R78" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S78" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="79" ht="42" customHeight="1">
       <x:c r="A79" s="51" t="str">
@@ -4602,9 +4350,6 @@
       <x:c r="R79" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S79" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="80" ht="42" customHeight="1">
       <x:c r="A80" s="51" t="str">
@@ -4651,9 +4396,6 @@
       <x:c r="R80" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S80" s="51" t="str">
-        <x:v>S07</x:v>
-      </x:c>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
       <x:c r="A81" s="51" t="str">
@@ -4700,9 +4442,6 @@
       <x:c r="R81" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S81" s="51" t="str">
-        <x:v>S01;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="82" ht="42" customHeight="1">
       <x:c r="A82" s="51" t="str">
@@ -4749,9 +4488,6 @@
       <x:c r="R82" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S82" s="51" t="str">
-        <x:v>S05;S06</x:v>
-      </x:c>
     </x:row>
     <x:row r="83" ht="42" customHeight="1">
       <x:c r="A83" s="51" t="str">
@@ -4798,9 +4534,6 @@
       <x:c r="R83" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S83" s="51" t="str">
-        <x:v>S05</x:v>
-      </x:c>
     </x:row>
     <x:row r="84" ht="42" customHeight="1">
       <x:c r="A84" s="51" t="str">
@@ -4847,9 +4580,6 @@
       <x:c r="R84" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S84" s="51" t="str">
-        <x:v>S05</x:v>
-      </x:c>
     </x:row>
     <x:row r="85" ht="42" customHeight="1">
       <x:c r="A85" s="51" t="str">
@@ -4896,9 +4626,6 @@
       <x:c r="R85" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S85" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="86" ht="42" customHeight="1">
       <x:c r="A86" s="51" t="str">
@@ -4945,9 +4672,6 @@
       <x:c r="R86" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S86" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="87" ht="42" customHeight="1">
       <x:c r="A87" s="51" t="str">
@@ -4994,9 +4718,6 @@
       <x:c r="R87" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S87" s="51" t="str">
-        <x:v>M01;S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="88" ht="42" customHeight="1">
       <x:c r="A88" s="51" t="str">
@@ -5043,9 +4764,6 @@
       <x:c r="R88" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S88" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="89" ht="42" customHeight="1">
       <x:c r="A89" s="51" t="str">
@@ -5092,9 +4810,6 @@
       <x:c r="R89" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S89" s="51" t="str">
-        <x:v>S01;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="90" ht="42" customHeight="1">
       <x:c r="A90" s="51" t="str">
@@ -5141,9 +4856,6 @@
       <x:c r="R90" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S90" s="51" t="str">
-        <x:v>S02;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="91" ht="42" customHeight="1">
       <x:c r="A91" s="51" t="str">
@@ -5190,9 +4902,6 @@
       <x:c r="R91" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S91" s="51" t="str">
-        <x:v>S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="92" ht="42" customHeight="1">
       <x:c r="A92" s="51" t="str">
@@ -5239,9 +4948,6 @@
       <x:c r="R92" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S92" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="93" ht="42" customHeight="1">
       <x:c r="A93" s="51" t="str">
@@ -5288,9 +4994,6 @@
       <x:c r="R93" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S93" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="94" ht="42" customHeight="1">
       <x:c r="A94" s="51" t="str">
@@ -5337,9 +5040,6 @@
       <x:c r="R94" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S94" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="95" ht="42" customHeight="1">
       <x:c r="A95" s="51" t="str">
@@ -5386,9 +5086,6 @@
       <x:c r="R95" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S95" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="96" ht="42" customHeight="1">
       <x:c r="A96" s="51" t="str">
@@ -5435,9 +5132,6 @@
       <x:c r="R96" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S96" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="97" ht="42" customHeight="1">
       <x:c r="A97" s="51" t="str">
@@ -5484,9 +5178,6 @@
       <x:c r="R97" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S97" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="98" ht="42" customHeight="1">
       <x:c r="A98" s="51" t="str">
@@ -5533,9 +5224,6 @@
       <x:c r="R98" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S98" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="99" ht="42" customHeight="1">
       <x:c r="A99" s="51" t="str">
@@ -5582,9 +5270,6 @@
       <x:c r="R99" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S99" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="100" ht="42" customHeight="1">
       <x:c r="A100" s="51" t="str">
@@ -5631,9 +5316,6 @@
       <x:c r="R100" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S100" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="101" ht="42" customHeight="1">
       <x:c r="A101" s="51" t="str">
@@ -5680,9 +5362,6 @@
       <x:c r="R101" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S101" s="51" t="str">
-        <x:v>S02;S04;M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="102" ht="42" customHeight="1">
       <x:c r="A102" s="51" t="str">
@@ -5729,9 +5408,6 @@
       <x:c r="R102" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S102" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="103" ht="42" customHeight="1">
       <x:c r="A103" s="51" t="str">
@@ -5778,9 +5454,6 @@
       <x:c r="R103" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S103" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="104" ht="42" customHeight="1">
       <x:c r="A104" s="51" t="str">
@@ -5827,9 +5500,6 @@
       <x:c r="R104" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S104" s="51" t="str">
-        <x:v>S02;S04</x:v>
-      </x:c>
     </x:row>
     <x:row r="105" ht="42" customHeight="1">
       <x:c r="A105" s="51" t="str">
@@ -5876,9 +5546,6 @@
       <x:c r="R105" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S105" s="51" t="str">
-        <x:v>M01;S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="106" ht="42" customHeight="1">
       <x:c r="A106" s="51" t="str">
@@ -5925,9 +5592,6 @@
       <x:c r="R106" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S106" s="51" t="str">
-        <x:v>S02;S03</x:v>
-      </x:c>
     </x:row>
     <x:row r="107" ht="42" customHeight="1">
       <x:c r="A107" s="51" t="str">
@@ -5974,9 +5638,6 @@
       <x:c r="R107" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S107" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="108" ht="42" customHeight="1">
       <x:c r="A108" s="51" t="str">
@@ -6023,9 +5684,6 @@
       <x:c r="R108" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S108" s="51" t="str">
-        <x:v>M01;S02</x:v>
-      </x:c>
     </x:row>
     <x:row r="109" ht="42" customHeight="1">
       <x:c r="A109" s="51" t="str">
@@ -6072,9 +5730,6 @@
       <x:c r="R109" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S109" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="110" ht="42" customHeight="1">
       <x:c r="A110" s="51" t="str">
@@ -6121,9 +5776,6 @@
       <x:c r="R110" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S110" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="111" ht="42" customHeight="1">
       <x:c r="A111" s="51" t="str">
@@ -6170,9 +5822,6 @@
       <x:c r="R111" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S111" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="112" ht="42" customHeight="1">
       <x:c r="A112" s="51" t="str">
@@ -6219,9 +5868,6 @@
       <x:c r="R112" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S112" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="113" ht="42" customHeight="1">
       <x:c r="A113" s="51" t="str">
@@ -6268,9 +5914,6 @@
       <x:c r="R113" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S113" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="114" ht="42" customHeight="1">
       <x:c r="A114" s="51" t="str">
@@ -6317,9 +5960,6 @@
       <x:c r="R114" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S114" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="115" ht="42" customHeight="1">
       <x:c r="A115" s="51" t="str">
@@ -6366,9 +6006,6 @@
       <x:c r="R115" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S115" s="51" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
     <x:row r="116" ht="42" customHeight="1">
       <x:c r="A116" s="51" t="str">
@@ -6415,9 +6052,6 @@
       <x:c r="R116" s="51" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S116" s="51" t="str">
-        <x:v>M01;S01</x:v>
-      </x:c>
     </x:row>
     <x:row r="117" ht="42" customHeight="1">
       <x:c r="A117" s="52" t="str">
@@ -6464,14 +6098,11 @@
       <x:c r="R117" s="52" t="str">
         <x:v>Keep</x:v>
       </x:c>
-      <x:c r="S117" s="52" t="str">
-        <x:v>M01</x:v>
-      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:S2"/>
-    <x:mergeCell ref="A3:S3"/>
+    <x:mergeCell ref="A2:R2"/>
+    <x:mergeCell ref="A3:R3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="M6:M117">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Complete"/>
@@ -6497,7 +6128,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74903552e6ad4226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3393d0ee62844440"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7010,7 +6641,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R284fbc847dd5417c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4a75f80efbf4c0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8051,232 +7682,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0df33118a92405d"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetPr>
-    <x:tabColor rgb="FF1A1A18"/>
-  </x:sheetPr>
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="2" t="str">
-        <x:v>Diligence Sources</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="18" customHeight="1">
-      <x:c r="A3" s="4" t="str">
-        <x:v>Source register — URLs and access dates are included for auditability.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="5"/>
-      <x:c r="B4" s="5"/>
-      <x:c r="C4" s="5"/>
-      <x:c r="D4" s="5"/>
-      <x:c r="E4" s="5"/>
-      <x:c r="F4" s="5"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="50" t="str">
-        <x:v>Source ID</x:v>
-      </x:c>
-      <x:c r="B5" s="50" t="str">
-        <x:v>Organization</x:v>
-      </x:c>
-      <x:c r="C5" s="50" t="str">
-        <x:v>Resource</x:v>
-      </x:c>
-      <x:c r="D5" s="50" t="str">
-        <x:v>Accessed</x:v>
-      </x:c>
-      <x:c r="E5" s="50" t="str">
-        <x:v>URL</x:v>
-      </x:c>
-      <x:c r="F5" s="50" t="str">
-        <x:v>Use in this workbook</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="51" t="str">
-        <x:v>S01</x:v>
-      </x:c>
-      <x:c r="B6" s="51" t="str">
-        <x:v>Deloitte</x:v>
-      </x:c>
-      <x:c r="C6" s="51" t="str">
-        <x:v>M&amp;A: The Intersection of Due Diligence and Governance</x:v>
-      </x:c>
-      <x:c r="D6" s="51" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E6" s="53" t="str">
-        <x:v>https://www.deloitte.com/us/en/programs/center-for-board-effectiveness/articles/mergers-and-acquisitions-due-diligence-and-governance.html</x:v>
-      </x:c>
-      <x:c r="F6" s="51" t="str">
-        <x:v>Core diligence workstreams; governance; operational diligence</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="51" t="str">
-        <x:v>S02</x:v>
-      </x:c>
-      <x:c r="B7" s="51" t="str">
-        <x:v>Deloitte</x:v>
-      </x:c>
-      <x:c r="C7" s="51" t="str">
-        <x:v>Prepare and execute the deal: Due diligence</x:v>
-      </x:c>
-      <x:c r="D7" s="51" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E7" s="53" t="str">
-        <x:v>https://www.deloitte.com/nl/en/Industries/tmt/perspectives/due-diligence.html</x:v>
-      </x:c>
-      <x:c r="F7" s="51" t="str">
-        <x:v>Integrated diligence; value, risk, synergies, integration handoff</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="51" t="str">
-        <x:v>S03</x:v>
-      </x:c>
-      <x:c r="B8" s="51" t="str">
-        <x:v>EY</x:v>
-      </x:c>
-      <x:c r="C8" s="51" t="str">
-        <x:v>M&amp;A Due Diligence Consulting Services</x:v>
-      </x:c>
-      <x:c r="D8" s="51" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E8" s="53" t="str">
-        <x:v>https://www.ey.com/en_in/services/strategy-transactions/mergers-acquisitions-due-diligence</x:v>
-      </x:c>
-      <x:c r="F8" s="51" t="str">
-        <x:v>Financial, commercial, operational, tax, cyber and Day 1 scope</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="51" t="str">
-        <x:v>S04</x:v>
-      </x:c>
-      <x:c r="B9" s="51" t="str">
-        <x:v>EY</x:v>
-      </x:c>
-      <x:c r="C9" s="51" t="str">
-        <x:v>Why due diligence has become vital to value creation</x:v>
-      </x:c>
-      <x:c r="D9" s="51" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E9" s="53" t="str">
-        <x:v>https://www.ey.com/en_gl/insights/private-equity/why-due-diligence-has-become-vital-to-value-creation</x:v>
-      </x:c>
-      <x:c r="F9" s="51" t="str">
-        <x:v>Diligence as value-creation work, not only risk identification</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="51" t="str">
-        <x:v>S05</x:v>
-      </x:c>
-      <x:c r="B10" s="51" t="str">
-        <x:v>FTC</x:v>
-      </x:c>
-      <x:c r="C10" s="51" t="str">
-        <x:v>Premerger Notification Program</x:v>
-      </x:c>
-      <x:c r="D10" s="51" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E10" s="53" t="str">
-        <x:v>https://www.ftc.gov/enforcement/premerger-notification-program</x:v>
-      </x:c>
-      <x:c r="F10" s="51" t="str">
-        <x:v>Current HSR process and resources; confirm applicability with counsel</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="51" t="str">
-        <x:v>S06</x:v>
-      </x:c>
-      <x:c r="B11" s="51" t="str">
-        <x:v>FTC</x:v>
-      </x:c>
-      <x:c r="C11" s="51" t="str">
-        <x:v>2026 HSR Threshold Update</x:v>
-      </x:c>
-      <x:c r="D11" s="51" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E11" s="53" t="str">
-        <x:v>https://www.ftc.gov/news-events/news/press-releases/2026/01/ftc-announces-2026-update-jurisdictional-fee-thresholds-premerger-notification-filings</x:v>
-      </x:c>
-      <x:c r="F11" s="51" t="str">
-        <x:v>Current thresholds change annually; do not rely on a stale hard-coded number</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="51" t="str">
-        <x:v>S07</x:v>
-      </x:c>
-      <x:c r="B12" s="51" t="str">
-        <x:v>DOJ / SEC</x:v>
-      </x:c>
-      <x:c r="C12" s="51" t="str">
-        <x:v>A Resource Guide to the U.S. Foreign Corrupt Practices Act</x:v>
-      </x:c>
-      <x:c r="D12" s="51" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E12" s="53" t="str">
-        <x:v>https://www.justice.gov/iso/opa/resources/29520121114101438198031.pdf</x:v>
-      </x:c>
-      <x:c r="F12" s="51" t="str">
-        <x:v>Anti-corruption diligence and successor-liability considerations</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="42" customHeight="1">
-      <x:c r="A13" s="52" t="str">
-        <x:v>M01</x:v>
-      </x:c>
-      <x:c r="B13" s="52" t="str">
-        <x:v>Mike Ye</x:v>
-      </x:c>
-      <x:c r="C13" s="52" t="str">
-        <x:v>Acquisition Lens Judgment Doctrine</x:v>
-      </x:c>
-      <x:c r="D13" s="52" t="str">
-        <x:v>2026-09-09</x:v>
-      </x:c>
-      <x:c r="E13" s="54" t="str">
-        <x:v>Internal MikeYe.com doctrine repository</x:v>
-      </x:c>
-      <x:c r="F13" s="52" t="str">
-        <x:v>Underwrite rather than admire; evidence, transferability, downside, structure and decision framing</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A3:F3"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra28db8cb6a5340f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re386bcf9a3cb469a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>